<commit_message>
Enhance Excel export: table, hyperlinks, number formats, timestamps
- Metadata banner row: lead count + generation timestamp
- Excel Table with filter dropdowns on every column
- LinkedIn, Website, Email → clickable hyperlinks
- Avg Rating → 0.0 format, Review Count → #,##0 with commas
- Level column: level1/level2 → Senior (L1) / Mid (L2)
- Exported At column with human-readable timestamp
- Freeze panes below metadata + header row

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Outputs/final_leads.xlsx
+++ b/Outputs/final_leads.xlsx
@@ -16,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,15 +33,29 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <color rgb="001155CC"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D2137"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -83,15 +99,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -168,6 +205,27 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LeadsTable" displayName="LeadsTable" ref="A2:L10" headerRowCount="1">
+  <autoFilter ref="A2:L10"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="Contact Name"/>
+    <tableColumn id="2" name="Title"/>
+    <tableColumn id="3" name="Level"/>
+    <tableColumn id="4" name="Email"/>
+    <tableColumn id="5" name="LinkedIn"/>
+    <tableColumn id="6" name="Company"/>
+    <tableColumn id="7" name="Website"/>
+    <tableColumn id="8" name="Address"/>
+    <tableColumn id="9" name="Phone"/>
+    <tableColumn id="10" name="Avg Rating"/>
+    <tableColumn id="11" name="Review Count"/>
+    <tableColumn id="12" name="Exported At"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -454,17 +512,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
@@ -473,134 +531,98 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>SortMyPrep Leads Export   |   8 leads   |   Generated: 07 May 2026, 02:38 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Contact Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Avg Rating</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Review Count</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Salih Veettil</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Founder and CEO</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>level1</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/salih-cheriya-veettil-751664324</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Edugravity Learning Centre</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>edugravity.com</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Al Reem Plaza - 107 Corniche St - Al Majaz 1 - Al Majaz - Sharjah - United Arab Emirates</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>+971 58 585 5199</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>59</v>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Exported At</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Hardik Tandel</t>
+          <t>Salih Veettil</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Head of Physics department</t>
+          <t>Founder and CEO</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>level2</t>
+          <t>Senior (L1)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/hardik-tandel-660827287</t>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/salih-cheriya-veettil-751664324</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -623,300 +645,405 @@
           <t>+971 58 585 5199</t>
         </is>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="J3" s="5" t="n">
         <v>4.9</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="K3" s="6" t="n">
         <v>59</v>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>07 May 2026, 02:38 AM</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Muhammed Nadeer</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Head of Academics</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>level2</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/muhammed-nadeer-b3292418b</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Hardik Tandel</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Head of Physics department</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Mid (L2)</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/hardik-tandel-660827287</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Edugravity Learning Centre</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>edugravity.com</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Al Reem Plaza - 107 Corniche St - Al Majaz 1 - Al Majaz - Sharjah - United Arab Emirates</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>+971 58 585 5199</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="9" t="n">
         <v>4.9</v>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="K4" s="10" t="n">
         <v>59</v>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>07 May 2026, 02:38 AM</t>
+        </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Jesna H</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Founder and Mathematics tutor</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>level1</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/jesna-k-h-84b94a122</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Jesnas Virtual Learning Hub</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Muwaileh Commercial - SPC Free Zone - Sharjah - United Arab Emirates</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>+971 55 465 6892</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>71</v>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Muhammed Nadeer</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Head of Academics</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Mid (L2)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/muhammed-nadeer-b3292418b</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Edugravity Learning Centre</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>edugravity.com</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Al Reem Plaza - 107 Corniche St - Al Majaz 1 - Al Majaz - Sharjah - United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>+971 58 585 5199</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>59</v>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>07 May 2026, 02:38 AM</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Abidah Quazeem</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>English Instructor</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>level1</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/abidah-quazeem-08581a198</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Jesna H</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Founder and Mathematics tutor</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Senior (L1)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jesna-k-h-84b94a122</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Jesnas Virtual Learning Hub</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Muwaileh Commercial - SPC Free Zone - Sharjah - United Arab Emirates</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>+971 55 465 6892</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="6" t="n">
         <v>71</v>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>07 May 2026, 02:38 AM</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Saida Rzayeva</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>level1</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/saida-rzayeva-66bb3325</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Progress Training Center</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>progresstraining.ae</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Al Majaz 2 - Al Majaz - Sharjah - United Arab Emirates</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>+971 50 232 1096</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>97</v>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Abidah Quazeem</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>English Instructor</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Senior (L1)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/abidah-quazeem-08581a198</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Jesnas Virtual Learning Hub</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Muwaileh Commercial - SPC Free Zone - Sharjah - United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>+971 55 465 6892</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>07 May 2026, 02:38 AM</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Syed Zahid</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Managing Director</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>level1</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/syed-zahid-97925542</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Saida Rzayeva</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Senior (L1)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/saida-rzayeva-66bb3325</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Progress Training Center</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>progresstraining.ae</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Al Majaz 2 - Al Majaz - Sharjah - United Arab Emirates</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>+971 50 232 1096</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="5" t="n">
         <v>4.8</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="6" t="n">
         <v>97</v>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>07 May 2026, 02:38 AM</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Syed Zahid</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Senior (L1)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/syed-zahid-97925542</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Progress Training Center</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>progresstraining.ae</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Al Majaz 2 - Al Majaz - Sharjah - United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>+971 50 232 1096</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>97</v>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>07 May 2026, 02:38 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
           <t>Muhammad Nuriddinov</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>SMM Manager</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>level2</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Mid (L2)</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/muhammad-ali-nuriddinov-b489b927a</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Progress Training Center</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>progresstraining.ae</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Al Majaz 2 - Al Majaz - Sharjah - United Arab Emirates</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>+971 50 232 1096</t>
         </is>
       </c>
-      <c r="J9" s="3" t="n">
+      <c r="J10" s="9" t="n">
         <v>4.8</v>
       </c>
-      <c r="K9" s="3" t="n">
+      <c r="K10" s="10" t="n">
         <v>97</v>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>07 May 2026, 02:38 AM</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1"/>
+    <hyperlink ref="E4" r:id="rId2"/>
+    <hyperlink ref="E5" r:id="rId3"/>
+    <hyperlink ref="E6" r:id="rId4"/>
+    <hyperlink ref="E7" r:id="rId5"/>
+    <hyperlink ref="E8" r:id="rId6"/>
+    <hyperlink ref="E9" r:id="rId7"/>
+    <hyperlink ref="E10" r:id="rId8"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId9"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>